<commit_message>
refactor: reorganize web routes and enhance error handling
This update refactors the web routes for improved modularity and maintainability. Key changes include:

- Split the scheduling routes into multiple modules for better organization and clarity.
- Updated error handling by moving Flask error handlers to a dedicated module.
- Enhanced the UI with a new mode selection feature in the base template.
- Improved comments and documentation across various scripts for better understanding.

These changes aim to streamline the codebase and enhance the user experience by providing a more structured approach to routing and error management.
</commit_message>
<xml_diff>
--- a/templates_excel/人员设备关联.xlsx
+++ b/templates_excel/人员设备关联.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -427,6 +427,16 @@
           <t>设备编号</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>技能等级</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>主操设备</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -437,6 +447,16 @@
       <c r="B2" t="inlineStr">
         <is>
           <t>CNC-01</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>

</xml_diff>